<commit_message>
Remove obsolete files related to DSIZ project phases and git history, including branch lists, estimated phases, and local environment configurations.
</commit_message>
<xml_diff>
--- a/.cursor/_olds/info/dataset_routes.xlsx
+++ b/.cursor/_olds/info/dataset_routes.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI\_PROJECTS\MES_midex\.cursor\_olds\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A45949B-22FE-4438-A717-3570BC404546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8276A9-A8C7-4C2D-AD9E-51A90E7DD1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="21429" xr2:uid="{2BE5B4B2-0955-468F-9A0F-6D751129322A}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset_routes" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -51,9 +51,6 @@
     <t xml:space="preserve"> GECO Крем_гель для очистки рук тела и волос, 2 л, Картридж, Крышка </t>
   </si>
   <si>
-    <t xml:space="preserve"> 00-000931 </t>
-  </si>
-  <si>
     <t xml:space="preserve"> GECO Крем гидрофильный СП, 100 мл, Лам, Винт </t>
   </si>
   <si>
@@ -400,6 +397,9 @@
   </si>
   <si>
     <t>WC_CHZ_MANUAL_AREA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 00-000968 </t>
   </si>
 </sst>
 </file>
@@ -950,49 +950,49 @@
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="K1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
@@ -1006,13 +1006,13 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G2" s="2">
         <v>15000</v>
@@ -1021,7 +1021,7 @@
         <v>720</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K2" s="2">
         <v>2</v>
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
@@ -1044,13 +1044,13 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H3" s="2">
         <v>5000</v>
@@ -1059,7 +1059,7 @@
         <v>720</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K3" s="2">
         <v>1</v>
@@ -1079,13 +1079,13 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H4" s="2">
         <v>1000</v>
@@ -1094,7 +1094,7 @@
         <v>720</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K4" s="2">
         <v>1</v>
@@ -1114,22 +1114,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I5" s="2">
+        <v>720</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H5" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I5" s="2">
-        <v>720</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
@@ -1140,22 +1140,22 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="C6" s="2">
         <v>1</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G6" s="2">
         <v>15000</v>
@@ -1164,7 +1164,7 @@
         <v>720</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K6" s="2">
         <v>2</v>
@@ -1173,27 +1173,27 @@
         <v>2</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="C7" s="2">
         <v>2</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H7" s="2">
         <v>5000</v>
@@ -1202,7 +1202,7 @@
         <v>720</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K7" s="2">
         <v>1</v>
@@ -1213,22 +1213,22 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C8" s="2">
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G8" s="2">
         <v>15000</v>
@@ -1237,7 +1237,7 @@
         <v>720</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K8" s="2">
         <v>2</v>
@@ -1246,27 +1246,27 @@
         <v>2</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C9" s="2">
         <v>2</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H9" s="2">
         <v>5000</v>
@@ -1275,7 +1275,7 @@
         <v>720</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K9" s="2">
         <v>1</v>
@@ -1286,22 +1286,22 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C10" s="2">
         <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H10" s="2">
         <v>1000</v>
@@ -1310,7 +1310,7 @@
         <v>720</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K10" s="2">
         <v>1</v>
@@ -1321,31 +1321,31 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C11" s="2">
         <v>2</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I11" s="2">
+        <v>720</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H11" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I11" s="2">
-        <v>720</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K11" s="2">
         <v>1</v>
@@ -1356,22 +1356,22 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C12" s="2">
         <v>1</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G12" s="2">
         <v>15000</v>
@@ -1380,7 +1380,7 @@
         <v>720</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K12" s="2">
         <v>2</v>
@@ -1389,27 +1389,27 @@
         <v>2</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H13" s="2">
         <v>5000</v>
@@ -1418,7 +1418,7 @@
         <v>720</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K13" s="2">
         <v>1</v>
@@ -1429,22 +1429,22 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C14" s="2">
         <v>1</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G14" s="2">
         <v>15000</v>
@@ -1453,7 +1453,7 @@
         <v>720</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K14" s="2">
         <v>2</v>
@@ -1462,27 +1462,27 @@
         <v>2</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C15" s="2">
         <v>2</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H15" s="2">
         <v>5000</v>
@@ -1491,7 +1491,7 @@
         <v>720</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K15" s="2">
         <v>1</v>
@@ -1502,22 +1502,22 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C16" s="2">
         <v>1</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H16" s="2">
         <v>1000</v>
@@ -1526,7 +1526,7 @@
         <v>720</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K16" s="2">
         <v>1</v>
@@ -1537,31 +1537,31 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C17" s="2">
         <v>2</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I17" s="2">
+        <v>720</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H17" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I17" s="2">
-        <v>720</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K17" s="2">
         <v>1</v>
@@ -1572,22 +1572,22 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C18" s="2">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H18" s="2">
         <v>1000</v>
@@ -1596,7 +1596,7 @@
         <v>720</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K18" s="2">
         <v>1</v>
@@ -1610,31 +1610,31 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C19" s="2">
         <v>2</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I19" s="2">
+        <v>720</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H19" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I19" s="2">
-        <v>720</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K19" s="2">
         <v>1</v>
@@ -1648,22 +1648,22 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="C20" s="2">
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G20" s="2">
         <v>15000</v>
@@ -1672,7 +1672,7 @@
         <v>720</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K20" s="2">
         <v>2</v>
@@ -1681,27 +1681,27 @@
         <v>2</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="C21" s="2">
         <v>2</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H21" s="2">
         <v>5000</v>
@@ -1710,7 +1710,7 @@
         <v>720</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K21" s="2">
         <v>1</v>
@@ -1721,22 +1721,22 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="C22" s="2">
         <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G22" s="2">
         <v>15000</v>
@@ -1745,7 +1745,7 @@
         <v>720</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K22" s="2">
         <v>2</v>
@@ -1754,27 +1754,27 @@
         <v>2</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="C23" s="2">
         <v>2</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H23" s="2">
         <v>5000</v>
@@ -1783,7 +1783,7 @@
         <v>720</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K23" s="2">
         <v>1</v>
@@ -1794,22 +1794,22 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="C24" s="2">
         <v>1</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G24" s="2">
         <v>15000</v>
@@ -1818,7 +1818,7 @@
         <v>720</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K24" s="2">
         <v>2</v>
@@ -1827,27 +1827,27 @@
         <v>2</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="C25" s="2">
         <v>2</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H25" s="2">
         <v>5000</v>
@@ -1856,7 +1856,7 @@
         <v>720</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K25" s="2">
         <v>1</v>
@@ -1867,22 +1867,22 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="C26" s="2">
         <v>1</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G26" s="2">
         <v>15000</v>
@@ -1891,7 +1891,7 @@
         <v>720</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K26" s="2">
         <v>2</v>
@@ -1900,27 +1900,27 @@
         <v>2</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="C27" s="2">
         <v>2</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H27" s="2">
         <v>5000</v>
@@ -1929,7 +1929,7 @@
         <v>720</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K27" s="2">
         <v>1</v>
@@ -1940,22 +1940,22 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="C28" s="2">
         <v>1</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G28" s="2">
         <v>15000</v>
@@ -1964,7 +1964,7 @@
         <v>720</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K28" s="2">
         <v>2</v>
@@ -1973,27 +1973,27 @@
         <v>2</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="C29" s="2">
         <v>2</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H29" s="2">
         <v>5000</v>
@@ -2002,7 +2002,7 @@
         <v>720</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K29" s="2">
         <v>1</v>
@@ -2013,22 +2013,22 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="C30" s="2">
         <v>1</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H30" s="2">
         <v>1000</v>
@@ -2037,7 +2037,7 @@
         <v>720</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K30" s="2">
         <v>1</v>
@@ -2048,31 +2048,31 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="C31" s="2">
         <v>2</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F31" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H31" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I31" s="2">
+        <v>720</v>
+      </c>
+      <c r="J31" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H31" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I31" s="2">
-        <v>720</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K31" s="2">
         <v>1</v>
@@ -2083,22 +2083,22 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="C32" s="2">
         <v>1</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G32" s="2">
         <v>15000</v>
@@ -2107,7 +2107,7 @@
         <v>720</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K32" s="2">
         <v>2</v>
@@ -2116,27 +2116,27 @@
         <v>2</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="C33" s="2">
         <v>2</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H33" s="2">
         <v>5000</v>
@@ -2145,7 +2145,7 @@
         <v>720</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K33" s="2">
         <v>1</v>
@@ -2156,22 +2156,22 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C34" s="2">
         <v>1</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G34" s="2">
         <v>15000</v>
@@ -2180,7 +2180,7 @@
         <v>720</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K34" s="2">
         <v>2</v>
@@ -2189,27 +2189,27 @@
         <v>2</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C35" s="2">
         <v>2</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H35" s="2">
         <v>5000</v>
@@ -2218,7 +2218,7 @@
         <v>720</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K35" s="2">
         <v>1</v>
@@ -2229,22 +2229,22 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="C36" s="2">
         <v>1</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H36" s="2">
         <v>1000</v>
@@ -2253,7 +2253,7 @@
         <v>720</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K36" s="2">
         <v>1</v>
@@ -2264,31 +2264,31 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="C37" s="2">
         <v>2</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F37" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H37" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I37" s="2">
+        <v>720</v>
+      </c>
+      <c r="J37" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H37" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I37" s="2">
-        <v>720</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K37" s="2">
         <v>1</v>
@@ -2299,22 +2299,22 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="C38" s="2">
         <v>1</v>
       </c>
       <c r="D38" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G38" s="2">
         <v>15000</v>
@@ -2323,7 +2323,7 @@
         <v>720</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K38" s="2">
         <v>2</v>
@@ -2332,27 +2332,27 @@
         <v>2</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="C39" s="2">
         <v>2</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H39" s="2">
         <v>5000</v>
@@ -2361,7 +2361,7 @@
         <v>720</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K39" s="2">
         <v>1</v>
@@ -2372,22 +2372,22 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="C40" s="2">
         <v>1</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G40" s="2">
         <v>15000</v>
@@ -2396,7 +2396,7 @@
         <v>720</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K40" s="2">
         <v>2</v>
@@ -2405,27 +2405,27 @@
         <v>2</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="C41" s="2">
         <v>2</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H41" s="2">
         <v>5000</v>
@@ -2434,7 +2434,7 @@
         <v>720</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K41" s="2">
         <v>1</v>
@@ -2445,22 +2445,22 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="C42" s="2">
         <v>1</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H42" s="2">
         <v>1000</v>
@@ -2469,7 +2469,7 @@
         <v>720</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K42" s="2">
         <v>1</v>
@@ -2480,31 +2480,31 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="C43" s="2">
         <v>2</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F43" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H43" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I43" s="2">
+        <v>720</v>
+      </c>
+      <c r="J43" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H43" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I43" s="2">
-        <v>720</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K43" s="2">
         <v>1</v>
@@ -2515,22 +2515,22 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="C44" s="2">
         <v>1</v>
       </c>
       <c r="D44" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="F44" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G44" s="2">
         <v>15000</v>
@@ -2539,7 +2539,7 @@
         <v>720</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K44" s="2">
         <v>2</v>
@@ -2548,27 +2548,27 @@
         <v>2</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="C45" s="2">
         <v>2</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H45" s="2">
         <v>5000</v>
@@ -2577,7 +2577,7 @@
         <v>720</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K45" s="2">
         <v>1</v>
@@ -2588,22 +2588,22 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="C46" s="2">
         <v>1</v>
       </c>
       <c r="D46" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="F46" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G46" s="2">
         <v>15000</v>
@@ -2612,7 +2612,7 @@
         <v>720</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K46" s="2">
         <v>2</v>
@@ -2621,27 +2621,27 @@
         <v>2</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="C47" s="2">
         <v>2</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H47" s="2">
         <v>5000</v>
@@ -2650,7 +2650,7 @@
         <v>720</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K47" s="2">
         <v>1</v>
@@ -2661,22 +2661,22 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="C48" s="2">
         <v>1</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H48" s="2">
         <v>1000</v>
@@ -2685,7 +2685,7 @@
         <v>720</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K48" s="2">
         <v>1</v>
@@ -2696,31 +2696,31 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="C49" s="2">
         <v>2</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F49" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H49" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I49" s="2">
+        <v>720</v>
+      </c>
+      <c r="J49" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H49" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I49" s="2">
-        <v>720</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K49" s="2">
         <v>1</v>
@@ -2731,31 +2731,31 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="C50" s="2">
         <v>1</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F50" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G50" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I50" s="2">
+        <v>720</v>
+      </c>
+      <c r="J50" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G50" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I50" s="2">
-        <v>720</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K50" s="2">
         <v>4</v>
@@ -2764,30 +2764,30 @@
         <v>3</v>
       </c>
       <c r="M50" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N50" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N50" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="C51" s="2">
         <v>2</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H51" s="2">
         <v>5000</v>
@@ -2796,7 +2796,7 @@
         <v>720</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K51" s="2">
         <v>1</v>
@@ -2807,31 +2807,31 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="C52" s="2">
         <v>1</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F52" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G52" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I52" s="2">
+        <v>720</v>
+      </c>
+      <c r="J52" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G52" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I52" s="2">
-        <v>720</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K52" s="2">
         <v>4</v>
@@ -2840,30 +2840,30 @@
         <v>3</v>
       </c>
       <c r="M52" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N52" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N52" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="C53" s="2">
         <v>2</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H53" s="2">
         <v>5000</v>
@@ -2872,7 +2872,7 @@
         <v>720</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K53" s="2">
         <v>1</v>
@@ -2883,22 +2883,22 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="C54" s="2">
         <v>1</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H54" s="2">
         <v>1000</v>
@@ -2907,7 +2907,7 @@
         <v>720</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K54" s="2">
         <v>1</v>
@@ -2918,31 +2918,31 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="C55" s="2">
         <v>2</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F55" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H55" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I55" s="2">
+        <v>720</v>
+      </c>
+      <c r="J55" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H55" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I55" s="2">
-        <v>720</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K55" s="2">
         <v>1</v>
@@ -2953,31 +2953,31 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="C56" s="2">
         <v>1</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G56" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I56" s="2">
+        <v>720</v>
+      </c>
+      <c r="J56" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G56" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I56" s="2">
-        <v>720</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K56" s="2">
         <v>4</v>
@@ -2986,30 +2986,30 @@
         <v>3</v>
       </c>
       <c r="M56" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N56" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="C57" s="2">
         <v>2</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H57" s="2">
         <v>5000</v>
@@ -3018,7 +3018,7 @@
         <v>720</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K57" s="2">
         <v>1</v>
@@ -3029,31 +3029,31 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A58" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="C58" s="2">
         <v>1</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F58" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G58" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I58" s="2">
+        <v>720</v>
+      </c>
+      <c r="J58" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G58" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I58" s="2">
-        <v>720</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K58" s="2">
         <v>4</v>
@@ -3062,30 +3062,30 @@
         <v>3</v>
       </c>
       <c r="M58" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N58" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A59" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="C59" s="2">
         <v>2</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H59" s="2">
         <v>5000</v>
@@ -3094,7 +3094,7 @@
         <v>720</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K59" s="2">
         <v>1</v>
@@ -3105,22 +3105,22 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="C60" s="2">
         <v>1</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E60" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H60" s="2">
         <v>500</v>
@@ -3129,7 +3129,7 @@
         <v>720</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K60" s="2">
         <v>1</v>
@@ -3140,31 +3140,31 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A61" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="C61" s="2">
         <v>2</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F61" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H61" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I61" s="2">
+        <v>720</v>
+      </c>
+      <c r="J61" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H61" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I61" s="2">
-        <v>720</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K61" s="2">
         <v>1</v>
@@ -3175,31 +3175,31 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A62" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="C62" s="2">
         <v>1</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F62" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G62" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I62" s="2">
+        <v>720</v>
+      </c>
+      <c r="J62" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G62" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I62" s="2">
-        <v>720</v>
-      </c>
-      <c r="J62" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K62" s="2">
         <v>4</v>
@@ -3208,30 +3208,30 @@
         <v>3</v>
       </c>
       <c r="M62" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N62" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N62" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A63" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="C63" s="2">
         <v>2</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H63" s="2">
         <v>5000</v>
@@ -3240,7 +3240,7 @@
         <v>720</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K63" s="2">
         <v>1</v>
@@ -3251,22 +3251,22 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A64" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C64" s="2">
         <v>1</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H64" s="2">
         <v>1000</v>
@@ -3275,7 +3275,7 @@
         <v>720</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K64" s="2">
         <v>1</v>
@@ -3286,31 +3286,31 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A65" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C65" s="2">
         <v>2</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F65" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H65" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I65" s="2">
+        <v>720</v>
+      </c>
+      <c r="J65" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H65" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I65" s="2">
-        <v>720</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K65" s="2">
         <v>1</v>
@@ -3321,22 +3321,22 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A66" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="C66" s="2">
         <v>1</v>
       </c>
       <c r="D66" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E66" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G66" s="2">
         <v>9000</v>
@@ -3345,7 +3345,7 @@
         <v>720</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K66" s="2">
         <v>2</v>
@@ -3354,27 +3354,27 @@
         <v>2</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A67" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="C67" s="2">
         <v>2</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H67" s="2">
         <v>5000</v>
@@ -3383,7 +3383,7 @@
         <v>720</v>
       </c>
       <c r="J67" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K67" s="2">
         <v>1</v>
@@ -3394,22 +3394,22 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A68" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B68" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C68" s="2">
         <v>1</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H68" s="2">
         <v>1000</v>
@@ -3418,7 +3418,7 @@
         <v>720</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K68" s="2">
         <v>1</v>
@@ -3429,31 +3429,31 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A69" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C69" s="2">
         <v>2</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F69" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H69" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I69" s="2">
+        <v>720</v>
+      </c>
+      <c r="J69" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H69" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I69" s="2">
-        <v>720</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K69" s="2">
         <v>1</v>
@@ -3464,22 +3464,22 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A70" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="C70" s="2">
         <v>1</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G70" s="2">
         <v>9000</v>
@@ -3488,7 +3488,7 @@
         <v>720</v>
       </c>
       <c r="J70" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K70" s="2">
         <v>2</v>
@@ -3497,27 +3497,27 @@
         <v>2</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A71" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="C71" s="2">
         <v>2</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H71" s="2">
         <v>5000</v>
@@ -3526,7 +3526,7 @@
         <v>720</v>
       </c>
       <c r="J71" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K71" s="2">
         <v>1</v>
@@ -3537,22 +3537,22 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A72" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B72" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="C72" s="2">
         <v>1</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H72" s="2">
         <v>1000</v>
@@ -3561,7 +3561,7 @@
         <v>720</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K72" s="2">
         <v>1</v>
@@ -3572,31 +3572,31 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A73" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B73" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="C73" s="2">
         <v>2</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F73" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H73" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I73" s="2">
+        <v>720</v>
+      </c>
+      <c r="J73" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H73" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I73" s="2">
-        <v>720</v>
-      </c>
-      <c r="J73" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="K73" s="2">
         <v>1</v>
@@ -3607,22 +3607,22 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A74" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="C74" s="2">
         <v>1</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G74" s="2">
         <v>9000</v>
@@ -3631,7 +3631,7 @@
         <v>720</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K74" s="2">
         <v>2</v>
@@ -3640,27 +3640,27 @@
         <v>2</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A75" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="C75" s="2">
         <v>2</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H75" s="2">
         <v>5000</v>
@@ -3669,7 +3669,7 @@
         <v>720</v>
       </c>
       <c r="J75" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K75" s="2">
         <v>1</v>
@@ -3680,22 +3680,22 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A76" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B76" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="C76" s="2">
         <v>1</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G76" s="2">
         <v>9000</v>
@@ -3704,7 +3704,7 @@
         <v>720</v>
       </c>
       <c r="J76" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K76" s="2">
         <v>2</v>
@@ -3713,27 +3713,27 @@
         <v>2</v>
       </c>
       <c r="N76" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A77" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B77" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="C77" s="2">
         <v>2</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H77" s="2">
         <v>5000</v>
@@ -3742,7 +3742,7 @@
         <v>720</v>
       </c>
       <c r="J77" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K77" s="2">
         <v>1</v>
@@ -3753,22 +3753,22 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A78" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B78" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="C78" s="2">
         <v>1</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G78" s="2">
         <v>7000</v>
@@ -3777,7 +3777,7 @@
         <v>720</v>
       </c>
       <c r="J78" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K78" s="2">
         <v>4</v>
@@ -3786,30 +3786,30 @@
         <v>3</v>
       </c>
       <c r="M78" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N78" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N78" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A79" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="C79" s="2">
         <v>2</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H79" s="2">
         <v>5000</v>
@@ -3818,7 +3818,7 @@
         <v>720</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K79" s="2">
         <v>1</v>
@@ -3829,31 +3829,31 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A80" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B80" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="C80" s="2">
         <v>1</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F80" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G80" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I80" s="2">
+        <v>720</v>
+      </c>
+      <c r="J80" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G80" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I80" s="2">
-        <v>720</v>
-      </c>
-      <c r="J80" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K80" s="2">
         <v>4</v>
@@ -3862,30 +3862,30 @@
         <v>3</v>
       </c>
       <c r="M80" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N80" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N80" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A81" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="C81" s="2">
         <v>2</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H81" s="2">
         <v>5000</v>
@@ -3894,7 +3894,7 @@
         <v>720</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K81" s="2">
         <v>1</v>
@@ -3905,22 +3905,22 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A82" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="C82" s="2">
         <v>1</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G82" s="2">
         <v>7000</v>
@@ -3929,7 +3929,7 @@
         <v>720</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K82" s="2">
         <v>4</v>
@@ -3938,30 +3938,30 @@
         <v>3</v>
       </c>
       <c r="M82" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N82" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N82" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="C83" s="2">
         <v>2</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H83" s="2">
         <v>5000</v>
@@ -3970,7 +3970,7 @@
         <v>720</v>
       </c>
       <c r="J83" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K83" s="2">
         <v>1</v>
@@ -3981,31 +3981,31 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A84" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="C84" s="2">
         <v>1</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F84" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G84" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I84" s="2">
+        <v>720</v>
+      </c>
+      <c r="J84" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G84" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I84" s="2">
-        <v>720</v>
-      </c>
-      <c r="J84" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="K84" s="2">
         <v>4</v>
@@ -4014,30 +4014,30 @@
         <v>3</v>
       </c>
       <c r="M84" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="N84" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="N84" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A85" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="C85" s="2">
         <v>2</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H85" s="2">
         <v>5000</v>
@@ -4046,7 +4046,7 @@
         <v>720</v>
       </c>
       <c r="J85" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K85" s="2">
         <v>1</v>
@@ -4057,22 +4057,22 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A86" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="C86" s="2">
         <v>1</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G86" s="2">
         <v>9000</v>
@@ -4081,7 +4081,7 @@
         <v>720</v>
       </c>
       <c r="J86" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K86" s="2">
         <v>2</v>
@@ -4090,27 +4090,27 @@
         <v>2</v>
       </c>
       <c r="N86" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A87" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B87" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="C87" s="2">
         <v>2</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H87" s="2">
         <v>5000</v>
@@ -4119,7 +4119,7 @@
         <v>720</v>
       </c>
       <c r="J87" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K87" s="2">
         <v>1</v>
@@ -4130,22 +4130,22 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A88" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B88" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="C88" s="2">
         <v>1</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G88" s="2">
         <v>9000</v>
@@ -4154,7 +4154,7 @@
         <v>720</v>
       </c>
       <c r="J88" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K88" s="2">
         <v>2</v>
@@ -4163,27 +4163,27 @@
         <v>2</v>
       </c>
       <c r="N88" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A89" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B89" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="C89" s="2">
         <v>2</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H89" s="2">
         <v>5000</v>
@@ -4192,7 +4192,7 @@
         <v>720</v>
       </c>
       <c r="J89" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K89" s="2">
         <v>1</v>

</xml_diff>